<commit_message>
fix(aset): menu Laporan pemeliharaan dan Laporan mutasi tidak lagi rusak
Kedua halaman laporan memanggil kode laporan yang tidak terdaftar, sehingga
pratinjau menjawab "laporan tidak dikenal" dan Cetak 404.

- Laporan pemeliharaan: definisi `laporan-pemeliharaan-aset` beserta layout
  bawaannya, melanjutkan PR #156. Lingkup unit kerja dan filter tambahan
  (K-30) mengikuti laporan aset lain.
- Laporan mutasi: halaman kini memakai laporan yang sudah terdaftar,
  `daftar-mutasi-aset` (alih-alih definisi kedua seperti di PR #150), dan
  layout serta definisinya dilengkapi untuk kolom yang dipakai layar.
- ReportScreenCodeTest membaca setiap layar module dan menolak kode laporan
  yang tidak terdaftar, supaya keadaan ini tidak sampai ke main lagi.

Co-Authored-By: Wisnu690 <wisnubagusindrayani@gmail.com>
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/daftar-mutasi-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/daftar-mutasi-aset/standar.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Mutasi aset" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mutasi aset'!$A$9:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mutasi aset'!$A$11:$O$11</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -65,6 +65,30 @@
   </si>
   <si>
     <t>${dicetak_pada}</t>
+  </si>
+  <si>
+    <t>Group aset</t>
+  </si>
+  <si>
+    <t>${filter_group}</t>
+  </si>
+  <si>
+    <t>Kelompok harta fiskal</t>
+  </si>
+  <si>
+    <t>${filter_golongan}</t>
+  </si>
+  <si>
+    <t>Jenis aset</t>
+  </si>
+  <si>
+    <t>${filter_jenis}</t>
+  </si>
+  <si>
+    <t>Aset</t>
+  </si>
+  <si>
+    <t>${filter_aset}</t>
   </si>
   <si>
     <t>Filter tambahan</t>
@@ -565,7 +589,7 @@
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="true" style="0"/>
@@ -690,103 +714,129 @@
       <c r="B8" t="s">
         <v>17</v>
       </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="J11" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="O9" s="6" t="s">
+      <c r="K11" s="6" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="L11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="F10" t="s">
+      <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="G10" t="s">
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="H10" t="s">
+      <c r="D12" t="s">
         <v>33</v>
       </c>
-      <c r="I10" t="s">
+      <c r="E12" t="s">
         <v>35</v>
       </c>
-      <c r="J10" t="s">
+      <c r="F12" t="s">
         <v>37</v>
       </c>
-      <c r="K10" t="s">
+      <c r="G12" t="s">
         <v>39</v>
       </c>
-      <c r="L10" t="s">
+      <c r="H12" t="s">
         <v>41</v>
       </c>
-      <c r="M10" t="s">
+      <c r="I12" t="s">
         <v>43</v>
       </c>
-      <c r="N10" t="s">
+      <c r="J12" t="s">
         <v>45</v>
       </c>
-      <c r="O10" t="s">
+      <c r="K12" t="s">
         <v>47</v>
       </c>
+      <c r="L12" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" t="s">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A9:O9"/>
+  <autoFilter ref="A11:O11"/>
   <mergeCells>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:N1"/>

</xml_diff>

<commit_message>
fix(aset): menu Laporan pemeliharaan dan Laporan mutasi tidak lagi rusak (#263)
Kedua halaman laporan memanggil kode laporan yang tidak terdaftar, sehingga
pratinjau menjawab "laporan tidak dikenal" dan Cetak 404.

- Laporan pemeliharaan: definisi `laporan-pemeliharaan-aset` beserta layout
  bawaannya, melanjutkan PR #156. Lingkup unit kerja dan filter tambahan
  (K-30) mengikuti laporan aset lain.
- Laporan mutasi: halaman kini memakai laporan yang sudah terdaftar,
  `daftar-mutasi-aset` (alih-alih definisi kedua seperti di PR #150), dan
  layout serta definisinya dilengkapi untuk kolom yang dipakai layar.
- ReportScreenCodeTest membaca setiap layar module dan menolak kode laporan
  yang tidak terdaftar, supaya keadaan ini tidak sampai ke main lagi.

Co-authored-by: Wisnu690 <wisnubagusindrayani@gmail.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/daftar-mutasi-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/daftar-mutasi-aset/standar.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Mutasi aset" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mutasi aset'!$A$9:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mutasi aset'!$A$11:$O$11</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -65,6 +65,30 @@
   </si>
   <si>
     <t>${dicetak_pada}</t>
+  </si>
+  <si>
+    <t>Group aset</t>
+  </si>
+  <si>
+    <t>${filter_group}</t>
+  </si>
+  <si>
+    <t>Kelompok harta fiskal</t>
+  </si>
+  <si>
+    <t>${filter_golongan}</t>
+  </si>
+  <si>
+    <t>Jenis aset</t>
+  </si>
+  <si>
+    <t>${filter_jenis}</t>
+  </si>
+  <si>
+    <t>Aset</t>
+  </si>
+  <si>
+    <t>${filter_aset}</t>
   </si>
   <si>
     <t>Filter tambahan</t>
@@ -565,7 +589,7 @@
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="true" style="0"/>
@@ -690,103 +714,129 @@
       <c r="B8" t="s">
         <v>17</v>
       </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="J11" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="O9" s="6" t="s">
+      <c r="K11" s="6" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="L11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="F10" t="s">
+      <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="G10" t="s">
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="H10" t="s">
+      <c r="D12" t="s">
         <v>33</v>
       </c>
-      <c r="I10" t="s">
+      <c r="E12" t="s">
         <v>35</v>
       </c>
-      <c r="J10" t="s">
+      <c r="F12" t="s">
         <v>37</v>
       </c>
-      <c r="K10" t="s">
+      <c r="G12" t="s">
         <v>39</v>
       </c>
-      <c r="L10" t="s">
+      <c r="H12" t="s">
         <v>41</v>
       </c>
-      <c r="M10" t="s">
+      <c r="I12" t="s">
         <v>43</v>
       </c>
-      <c r="N10" t="s">
+      <c r="J12" t="s">
         <v>45</v>
       </c>
-      <c r="O10" t="s">
+      <c r="K12" t="s">
         <v>47</v>
       </c>
+      <c r="L12" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" t="s">
+        <v>55</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A9:O9"/>
+  <autoFilter ref="A11:O11"/>
   <mergeCells>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:N1"/>

</xml_diff>